<commit_message>
+V2 : refactor with UI
</commit_message>
<xml_diff>
--- a/02.Config/config.xlsx
+++ b/02.Config/config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03.Dev\01.Project\02.AttendanceServer\02.Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA43B2A8-F71C-40FE-94D1-4EF76BBE829D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF9FBC3-D4BF-4C8B-93E8-4DE5F3A04792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6354BC04-B487-417A-81BA-EC62C1F93913}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -79,9 +79,6 @@
     <t>ot_folder</t>
   </si>
   <si>
-    <t>mang thai</t>
-  </si>
-  <si>
     <t>Con nhỏ dưới 12 tháng</t>
   </si>
   <si>
@@ -154,9 +151,6 @@
     <t>\\10.0.1.5\tiqn\03.Department\01.Operation Management\03.HR-GA\01.HR\7 Resigned list\Resigned report.xlsx</t>
   </si>
   <si>
-    <t>\\10.0.1.5\tiqn\03.Department\01.Operation Management\03.HR-GA\05.Nurse\5. Maternity leave\Danh sách nhân viên nữ mang thai.xlsx</t>
-  </si>
-  <si>
     <t>\\10.0.1.5\tiqn\03.Department\01.Operation Management\03.HR-GA\01.HR\4. EMPLOYEE\7.OT request</t>
   </si>
   <si>
@@ -170,6 +164,21 @@
   </si>
   <si>
     <t>10.0.1.44</t>
+  </si>
+  <si>
+    <t>\\10.0.1.5\tiqn\03.Department\01.Operation Management\03.HR-GA\05.Nurse\5. Maternity leave\Danh sách nhân viên nữ mang thai 1.xlsx</t>
+  </si>
+  <si>
+    <t>Mang thai</t>
+  </si>
+  <si>
+    <t>10.0.1.45</t>
+  </si>
+  <si>
+    <t>10.0.1.46</t>
+  </si>
+  <si>
+    <t>10.0.1.47</t>
   </si>
 </sst>
 </file>
@@ -386,8 +395,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2CBE66FE-8037-4834-BA52-F066E6D20D2F}" name="Table1" displayName="Table1" ref="A1:B5" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:B5" xr:uid="{2CBE66FE-8037-4834-BA52-F066E6D20D2F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2CBE66FE-8037-4834-BA52-F066E6D20D2F}" name="Table1" displayName="Table1" ref="A1:B8" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:B8" xr:uid="{2CBE66FE-8037-4834-BA52-F066E6D20D2F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{2EB51117-8229-4C78-AC8D-8813DD389044}" name="No" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{10A8DD70-50F7-4EA6-A521-606C4ADB9982}" name="IP" dataDxfId="0"/>
@@ -740,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38EBA017-E946-45D2-9470-ABE41CCBB9FA}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.296875" customWidth="1"/>
@@ -759,7 +768,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -767,7 +776,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -775,7 +784,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -783,7 +792,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -824,7 +857,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -835,7 +868,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -846,7 +879,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -857,60 +890,60 @@
         <v>7</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="5"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="\\192.168.1.13\tiqn\03.Department\01.Operation Management\03.HR-GA\01.HR\7 Resigned list\Resigned report.xlsx" xr:uid="{8F64EE08-73F5-4DA5-91C3-D424BA7B7DBD}"/>
-    <hyperlink ref="C4" r:id="rId2" display="\\192.168.1.13\tiqn\03.Department\01.Operation Management\03.HR-GA\05.Nurse\5. Maternity leave\Danh sách nhân viên nữ mang thai.xlsx" xr:uid="{B89DC985-5B7C-4536-B175-E107F8D3392B}"/>
+    <hyperlink ref="C4" r:id="rId2" xr:uid="{B89DC985-5B7C-4536-B175-E107F8D3392B}"/>
     <hyperlink ref="C2" r:id="rId3" display="\\192.168.1.13\tiqn\03.Department\01.Operation Management\03.HR-GA\01.HR\Toray's employees information All in one.xlsx" xr:uid="{62034D28-22E1-4E8D-8AE0-4315F4FEF4DB}"/>
     <hyperlink ref="C5" r:id="rId4" display="\\192.168.1.13\tiqn\03.Department\01.Operation Management\03.HR-GA\01.HR\4. EMPLOYEE\7.OT request" xr:uid="{06546D36-137D-428D-802B-892800614F10}"/>
   </hyperlinks>
@@ -933,10 +966,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -947,10 +980,10 @@
         <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -958,10 +991,10 @@
         <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -969,10 +1002,10 @@
         <v>161</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -980,10 +1013,10 @@
         <v>623</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -991,10 +1024,10 @@
         <v>916</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1002,10 +1035,10 @@
         <v>920</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>